<commit_message>
Add excel parser service
</commit_message>
<xml_diff>
--- a/backend/testdata/zobaroute_testfile_v1.xlsx
+++ b/backend/testdata/zobaroute_testfile_v1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/28702308897aee29/Studium/Diplomarbeit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\zobaroute\backend\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_79DADAAF517A1A9EED329076445DCE3AA7C83915" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95CCBA62-6082-4149-8A0A-31E190143A7B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648A3BBB-E8A7-49F9-A768-B6302AF70C28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bestellungen" sheetId="1" r:id="rId1"/>
@@ -268,15 +268,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -585,19 +582,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="13" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="9.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.1796875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,7 +623,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -636,7 +633,7 @@
       <c r="C2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>8472</v>
       </c>
       <c r="E2" s="2" t="s">
@@ -651,7 +648,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
@@ -661,7 +658,7 @@
       <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>8472</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -678,7 +675,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -688,7 +685,7 @@
       <c r="C4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>8472</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -701,7 +698,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -711,7 +708,7 @@
       <c r="C5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>8404</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -724,7 +721,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
@@ -734,7 +731,7 @@
       <c r="C6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>8404</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -749,7 +746,7 @@
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
@@ -759,7 +756,7 @@
       <c r="C7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>8472</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -774,7 +771,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>31</v>
       </c>
@@ -784,7 +781,7 @@
       <c r="C8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>8472</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -799,7 +796,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
         <v>34</v>
@@ -807,7 +804,7 @@
       <c r="C9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>8472</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -822,7 +819,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>36</v>
       </c>
@@ -830,7 +827,7 @@
       <c r="C10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>8472</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -843,7 +840,7 @@
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>38</v>
       </c>
@@ -851,7 +848,7 @@
         <v>39</v>
       </c>
       <c r="C11" s="2"/>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>8472</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -864,7 +861,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
@@ -887,7 +884,7 @@
       </c>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>43</v>
       </c>
@@ -897,7 +894,7 @@
       <c r="C13" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>8472</v>
       </c>
       <c r="E13" s="2"/>
@@ -908,7 +905,7 @@
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
@@ -918,7 +915,7 @@
       <c r="C14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <v>8472</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -933,7 +930,7 @@
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>46</v>
       </c>
@@ -943,7 +940,7 @@
       <c r="C15" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <v>8472</v>
       </c>
       <c r="E15" s="2" t="s">
@@ -956,7 +953,7 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>49</v>
       </c>
@@ -966,7 +963,7 @@
       <c r="C16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="2">
         <v>8472</v>
       </c>
       <c r="E16" s="2" t="s">
@@ -981,7 +978,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>52</v>
       </c>
@@ -991,7 +988,7 @@
       <c r="C17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>8472</v>
       </c>
       <c r="E17" s="2" t="s">
@@ -1008,7 +1005,7 @@
       </c>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>54</v>
       </c>
@@ -1018,7 +1015,7 @@
       <c r="C18" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="2">
         <v>8472</v>
       </c>
       <c r="E18" s="2" t="s">
@@ -1033,7 +1030,7 @@
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>56</v>
       </c>
@@ -1043,7 +1040,7 @@
       <c r="C19" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="2">
         <v>8472</v>
       </c>
       <c r="E19" s="2" t="s">
@@ -1056,7 +1053,7 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>59</v>
       </c>
@@ -1066,7 +1063,7 @@
       <c r="C20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="2">
         <v>8472</v>
       </c>
       <c r="E20" s="2" t="s">
@@ -1079,7 +1076,7 @@
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>63</v>
       </c>
@@ -1089,7 +1086,7 @@
       <c r="C21" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
         <v>8472</v>
       </c>
       <c r="E21" s="2" t="s">

</xml_diff>